<commit_message>
Update game data: new monsters, moves, traits, move pools, and validation scripts
</commit_message>
<xml_diff>
--- a/backend/data/data_stats_traits_formal.xlsx
+++ b/backend/data/data_stats_traits_formal.xlsx
@@ -1,26 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Alan\Github Projects\roco-kingdom-team-builder\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99951F79-2E5D-48B1-A290-893DDE59B7F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB1CB63A-AABA-4F7A-86E1-7CAE418FB828}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -63,7 +58,7 @@
     <t>草</t>
   </si>
   <si>
-    <t>系统发育: 获得能量或生命时,会将等量的能量或生命随机分配给场下的精灵。</t>
+    <t>系统发育：获得能量或生命时，会将等量的能量或生命随机分配给场下的精灵。</t>
   </si>
   <si>
     <t>粉耳星兔</t>
@@ -72,7 +67,7 @@
     <t>幻</t>
   </si>
   <si>
-    <t>双向光速: 在场时,所有回合结束时效果,触发次数+1。</t>
+    <t>双向光速：在场时，所有回合结束时效果，触发次数+1。</t>
   </si>
   <si>
     <t>落陨星兔</t>
@@ -81,7 +76,7 @@
     <t>幻 / 幽</t>
   </si>
   <si>
-    <t>陨落: 在场时,双方回合结束时触发的效果,触发次数-1。</t>
+    <t>陨落：在场时，双方回合结束时触发的效果，触发次数-1。</t>
   </si>
   <si>
     <t>贝古斯</t>
@@ -90,7 +85,7 @@
     <t>机械 / 火</t>
   </si>
   <si>
-    <t>贪心算法: 1号位技能获得传劲1,且使用后使敌方获得6层灼烧。</t>
+    <t>贪心算法：1号位技能获得传劲1，且使用后使敌方获得6层灼烧。</t>
   </si>
   <si>
     <t>小皮球</t>
@@ -99,7 +94,7 @@
     <t>电 / 幻</t>
   </si>
   <si>
-    <t>星地善良: 回合结束时,若场上的己方精灵能量等于0,自己立即替换此精灵</t>
+    <t>星地善良：回合结束时，若场上的己方精灵能量等于0，自己立即替换此精灵。</t>
   </si>
   <si>
     <t>夜枭</t>
@@ -108,16 +103,13 @@
     <t>幽</t>
   </si>
   <si>
-    <t>搜刮: 敌方每使用1次「聚能」技能或更换精灵,自己入场时获得魔攻+20%。</t>
-  </si>
-  <si>
     <t>燃薪虫</t>
   </si>
   <si>
     <t>火 / 草</t>
   </si>
   <si>
-    <t>煤渣草: 在场时,所有灼烧的衰减变为增长。</t>
+    <t>煤渣草：在场时，所有灼烧的衰减变为增长。</t>
   </si>
   <si>
     <t>窃光蚊</t>
@@ -126,7 +118,7 @@
     <t>恶 / 光</t>
   </si>
   <si>
-    <t>血型吸引: 敌方每携带1种系列的技能,自己攻击时威力+10。</t>
+    <t>血型吸引：敌方每携带1种系列的技能，自己攻击时威力+10。</t>
   </si>
   <si>
     <t>月牙雪熊</t>
@@ -135,7 +127,7 @@
     <t>冰 / 幻</t>
   </si>
   <si>
-    <t>月牙雪糕: 使用攻击技能时,敌方每层冻结视为1层额外星痕印记。</t>
+    <t>月牙雪糕：使用攻击技能时，敌方每层冻结视为1层额外星痕印记。</t>
   </si>
   <si>
     <t>利灯鱼</t>
@@ -144,7 +136,7 @@
     <t>水 / 电</t>
   </si>
   <si>
-    <t>对流: 自己的能耗增加变为能耗降低;能耗降低变为能耗增加。</t>
+    <t>对流：自己的能耗增加变为能耗降低；能耗降低变为能耗增加。</t>
   </si>
   <si>
     <t>陨星虫</t>
@@ -153,7 +145,7 @@
     <t>虫</t>
   </si>
   <si>
-    <t>契约的形状: 根据捕捉所用的咕噜球,入场时获得不同效果。</t>
+    <t>契约的形状：根据捕捉所用的咕噜球，入场时获得不同效果。</t>
   </si>
   <si>
     <t>熔岩布丁</t>
@@ -162,7 +154,7 @@
     <t>水 / 火</t>
   </si>
   <si>
-    <t>美拉德反应: 离场后,更换入场的精灵获得双攻+20%且免疫灼烧。</t>
+    <t>美拉德反应：离场后，更换入场的精灵获得双攻+20%且免疫灼烧。</t>
   </si>
   <si>
     <t>椰浆布丁</t>
@@ -171,7 +163,7 @@
     <t>水 / 冰</t>
   </si>
   <si>
-    <t>吉利丁片: 离场后,更换入场的精灵获得双防+20%且免疫冻结。</t>
+    <t>吉利丁片：离场后，更换入场的精灵获得双防+20%且免疫冻结。</t>
   </si>
   <si>
     <t>抹茶布丁</t>
@@ -180,7 +172,7 @@
     <t>水 / 草</t>
   </si>
   <si>
-    <t>茶多酚: 离场后,更换入场的精灵回复20%生命且免疫寄生。</t>
+    <t>茶多酚：离场后，更换入场的精灵回复20%生命且免疫寄生。</t>
   </si>
   <si>
     <t>疾光千兽</t>
@@ -189,7 +181,7 @@
     <t>光</t>
   </si>
   <si>
-    <t>月光审判: 攻击时,若敌方血脉是首领血脉,技能威力+100%。</t>
+    <t>月光审判：攻击时，若敌方血脉是首领血脉，技能威力+100%。</t>
   </si>
   <si>
     <t>绒仙子</t>
@@ -198,16 +190,16 @@
     <t>光 / 虫</t>
   </si>
   <si>
-    <t>缤纷星光: 攻击时,若敌方血脉是非本系的系列血脉,技能威力+100%。</t>
-  </si>
-  <si>
-    <t>古卷巨魔像</t>
+    <t>缤纷星光：攻击时，若敌方血脉是非本系的系列血脉，技能威力+100%。</t>
+  </si>
+  <si>
+    <t>古卷匣魔像</t>
   </si>
   <si>
     <t>普通 / 武</t>
   </si>
   <si>
-    <t>构装契约者: 入场时,若敌方魔力值为1,自己获得双防+50%。</t>
+    <t>构装契约者：入场时，若敌方魔力值为1，自己获得双防+50%。</t>
   </si>
   <si>
     <t>古卷执政官</t>
@@ -216,19 +208,19 @@
     <t>普通 / 幻</t>
   </si>
   <si>
-    <t>图书守卫者: 入场时,若自己魔力值为1,自己获得双攻+50%。</t>
+    <t>图书守卫者：入场时，若自己魔力值为1，自己获得双攻+50%。</t>
   </si>
   <si>
     <t>画间沉铁兽</t>
   </si>
   <si>
-    <t>变形活画: 攻击时,敌方每有1层增益,本次技能威力+10%。</t>
+    <t>变形活画：攻击时，敌方每有1层增益，本次技能威力+10%。</t>
   </si>
   <si>
     <t>画间法师手</t>
   </si>
   <si>
-    <t>灰色肖像: 攻击会摧毁敌方已有的减益层数+3。</t>
+    <t>灰色肖像：攻击会摧毁敌方已有的减益层数+3。</t>
   </si>
   <si>
     <t>食尘短绒</t>
@@ -237,13 +229,13 @@
     <t>虫 / 地</t>
   </si>
   <si>
-    <t>特殊清洁场景: 回合结束时偷取敌方1层印记。</t>
+    <t>特殊清洁场景：回合结束时偷取敌方1层印记。</t>
   </si>
   <si>
     <t>捕尘长绒</t>
   </si>
   <si>
-    <t>扫拖一体: 回合结束时驱散敌方1层印记,且驱散后己方队伍获得1次碰机奉献。</t>
+    <t>扫拖一体：回合结束时驱散敌方1层印记，且驱散后己方队伍获得1次碰机奉献。</t>
   </si>
   <si>
     <t>龙息帕尔</t>
@@ -252,16 +244,16 @@
     <t>冰 / 恶</t>
   </si>
   <si>
-    <t>付给恶魔的赎价: 击败敌方精灵时,敌方额外损失1点魔力。被敌方精灵击败时,自己额外损失1点魔力。</t>
-  </si>
-  <si>
-    <t>厉毒修罗</t>
+    <t>付给恶魔的赎价：击败敌方精灵时，敌方额外损失1点魔力。被敌方精灵击败时，自己额外损失1点魔力。</t>
+  </si>
+  <si>
+    <t>厉毒修萝</t>
   </si>
   <si>
     <t>毒 / 恶</t>
   </si>
   <si>
-    <t>侵蚀: 敌方每有1层中毒效果,自己获得连击数+1。</t>
+    <t>侵蚀：敌方每有1层中毒效果，自己获得连击数+1。</t>
   </si>
   <si>
     <t>寂灭骨龙</t>
@@ -270,7 +262,7 @@
     <t>龙 / 幽</t>
   </si>
   <si>
-    <t>不朽: 力量2回合后复活。</t>
+    <t>不朽：力量2回合后复活。</t>
   </si>
   <si>
     <t>泥吼牙</t>
@@ -279,7 +271,7 @@
     <t>地 / 翼</t>
   </si>
   <si>
-    <t>无差别过滤: 在场时,所有精灵连击数固定为2。</t>
+    <t>无差别过滤：在场时，所有精灵连击数固定为2。</t>
   </si>
   <si>
     <t>圣剑-X</t>
@@ -288,13 +280,13 @@
     <t>机械</t>
   </si>
   <si>
-    <t>正位宝剑: 仅可以使用1号位技能。</t>
+    <t>正位宝剑：仅可以使用1号位技能。</t>
   </si>
   <si>
     <t>铠甲虫</t>
   </si>
   <si>
-    <t>坚韧铠甲: 每受到1次攻击伤害,己方队伍获得1次随机奉献。</t>
+    <t>坚韧铠甲：每受到1次攻击伤害，己方队伍获得1次随机奉献。</t>
   </si>
   <si>
     <t>混乱鱿彩</t>
@@ -303,7 +295,7 @@
     <t>幽 / 恶</t>
   </si>
   <si>
-    <t>涂鸦: 使用非本系技能时威力+50%。</t>
+    <t>涂鸦：使用非本系技能时威力+50%。</t>
   </si>
   <si>
     <t>秩序鱿墨</t>
@@ -312,7 +304,7 @@
     <t>幽 / 萌</t>
   </si>
   <si>
-    <t>绝对秩序: 受到非敌方系列的技能攻击时伤害-50%。</t>
+    <t>绝对秩序：受到非敌方系列的技能攻击时伤害-50%。</t>
   </si>
   <si>
     <t>遁地鼠</t>
@@ -321,13 +313,13 @@
     <t>地</t>
   </si>
   <si>
-    <t>警惕: 回合结束时,若自己能量为0则逃离。</t>
+    <t>警惕：回合结束时，若自己能量为0则逃离。</t>
   </si>
   <si>
     <t>格兰球</t>
   </si>
   <si>
-    <t>生长: 回合结束时,回复12%生命。</t>
+    <t>生长：回合结束时，回复12%生命。</t>
   </si>
   <si>
     <t>深蓝鲸</t>
@@ -336,16 +328,16 @@
     <t>水</t>
   </si>
   <si>
-    <t>倾轧: 携带的技能受能耗变化效果的影响翻倍。</t>
-  </si>
-  <si>
-    <t>啪嗒鸟</t>
+    <t>倾轧：携带的技能受能耗变化效果的影响翻倍。</t>
+  </si>
+  <si>
+    <t>噼啪鸟</t>
   </si>
   <si>
     <t>电 / 翼</t>
   </si>
   <si>
-    <t>连续负荷: 自己技能的迸发效果延长1回合。</t>
+    <t>连续负荷：自己技能的迸发效果延长1回合。</t>
   </si>
   <si>
     <t>绒光优优</t>
@@ -354,7 +346,7 @@
     <t>地 / 光</t>
   </si>
   <si>
-    <t>哨兵: 回合开始时若敌方能足量击败自己,自己获得速度+50,行动后脱离。</t>
+    <t>哨兵：回合开始时若敌方能足量击败自己，自己获得速度+50，行动后脱离。</t>
   </si>
   <si>
     <t>武者鸡</t>
@@ -363,19 +355,19 @@
     <t>火 / 武</t>
   </si>
   <si>
-    <t>斗技: 应对成功后,获得全技能威力永久+20。</t>
+    <t>斗技：应对成功后，获得全技能威力永久+20。</t>
   </si>
   <si>
     <t>绅士鸡</t>
   </si>
   <si>
-    <t>指挥家: 应对成功后,永久获得双攻+20%。</t>
+    <t>指挥家：应对成功后，永久获得双攻+20%。</t>
   </si>
   <si>
     <t>立方人</t>
   </si>
   <si>
-    <t>盲拧: 回合开始时,技能顺序打乱,4号位的技能能耗-4。</t>
+    <t>盲拧：回合开始时，技能顺序打乱，4号位的技能能耗-4。</t>
   </si>
   <si>
     <t>帕帕斯卡</t>
@@ -384,7 +376,7 @@
     <t>机械 / 翼</t>
   </si>
   <si>
-    <t>翼轴: 1号位技能获得迅捷和传动1。</t>
+    <t>翼轴：1号位技能获得迅捷和传动1。</t>
   </si>
   <si>
     <t>乌拉塔</t>
@@ -393,7 +385,7 @@
     <t>恶 / 火</t>
   </si>
   <si>
-    <t>恶魔的晚宴: 主动击败敌方精灵时,自己获得双攻+50%。</t>
+    <t>恶魔的晚宴：主动击败敌方精灵时，自己获得双攻+50%。</t>
   </si>
   <si>
     <t>红绒十字</t>
@@ -402,7 +394,7 @@
     <t>火 / 萌</t>
   </si>
   <si>
-    <t>仁心: 敌方受到灼烧伤害时,自己回复等量生命。</t>
+    <t>仁心：敌方受到灼烧伤害时，自己回复等量生命。</t>
   </si>
   <si>
     <t>冰钻布鲁斯</t>
@@ -411,7 +403,7 @@
     <t>冰</t>
   </si>
   <si>
-    <t>冰钻: 敌方携带技能总能耗每有1点,自己攻击时威力+10%。</t>
+    <t>冰钻：敌方携带技能总能耗每有1点，自己攻击时威力+10%。</t>
   </si>
   <si>
     <t>火焰猿</t>
@@ -420,7 +412,7 @@
     <t>火</t>
   </si>
   <si>
-    <t>散热: 初始能量为0,入场前己方精灵每放1次火系技能,回复3能量。</t>
+    <t>散热：初始能量为0，入场前己方精灵每放1次火系技能，回复3能量。</t>
   </si>
   <si>
     <t>裘卡</t>
@@ -429,7 +421,7 @@
     <t>毒</t>
   </si>
   <si>
-    <t>蚀刻: 回合结束时,敌方每2层中毒转化为1层中毒印记。</t>
+    <t>蚀刻：回合结束时，敌方每2层中毒转化为1层中毒印记。</t>
   </si>
   <si>
     <t>琉璃水母</t>
@@ -438,7 +430,7 @@
     <t>水 / 毒</t>
   </si>
   <si>
-    <t>扩散侵蚀: 使用水系技能后,敌方获得中毒,获得层数等于中毒印记层数的2倍。</t>
+    <t>扩散侵蚀：使用水系技能后，敌方获得中毒，获得层数等于中毒印记层数的2倍。</t>
   </si>
   <si>
     <t>闪电鳗鱼</t>
@@ -447,13 +439,10 @@
     <t>电 / 水</t>
   </si>
   <si>
-    <t>生物电: 携带的电系技能获得迸发:能耗-2。</t>
-  </si>
-  <si>
     <t>圣代甜甜 (樱桃)</t>
   </si>
   <si>
-    <t>加个雪球: 使敌方获得冻结时,也会使其获得2层冻结。</t>
+    <t>加个雪球：使敌方获得冻结时，也会使其获得2层冻结。</t>
   </si>
   <si>
     <t>圣代甜甜 (抹茶)</t>
@@ -468,7 +457,7 @@
     <t>水 / 龙</t>
   </si>
   <si>
-    <t>洄游: 每次进入蓄力状态,获得全技能能耗永久-1。</t>
+    <t>洄游：每次进入蓄力状态，获得全技能能耗永久-1。</t>
   </si>
   <si>
     <t>月亮砣</t>
@@ -477,22 +466,22 @@
     <t>毒 / 萌</t>
   </si>
   <si>
-    <t>耐活王: 敌方受到中毒效果伤害时,自己回复等量生命。</t>
-  </si>
-  <si>
-    <t>高脚鹮</t>
+    <t>耐活王：敌方受到中毒效果伤害时，自己回复等量生命。</t>
+  </si>
+  <si>
+    <t>高脚鹬</t>
   </si>
   <si>
     <t>翼 / 冰</t>
   </si>
   <si>
-    <t>起飞加速: 本场战斗首次使用的技能获得迅捷。</t>
+    <t>起飞加速：本场战斗首次使用的技能获得迅捷。</t>
   </si>
   <si>
     <t>声波缇塔</t>
   </si>
   <si>
-    <t>向心力: 1号和2号位技能获得传动1和威力+30。</t>
+    <t>向心力：1号和2号位技能获得传动1和威力+30。</t>
   </si>
   <si>
     <t>爵士鹿</t>
@@ -501,7 +490,7 @@
     <t>电</t>
   </si>
   <si>
-    <t>蓄电池: 每入场1次,永久获得双攻+20%。</t>
+    <t>蓄电池：每入场1次，永久获得双攻+20%。</t>
   </si>
   <si>
     <t>海枝枝 (日冕)</t>
@@ -510,7 +499,7 @@
     <t>水 / 幽</t>
   </si>
   <si>
-    <t>珊瑚骨: 敌方精灵退场时,自己获得全技能能耗-3。</t>
+    <t>珊瑚骨：敌方精灵退场时，自己获得全技能能耗-3。</t>
   </si>
   <si>
     <t>海枝枝 (洋红)</t>
@@ -528,7 +517,7 @@
     <t>龙 / 翼</t>
   </si>
   <si>
-    <t>暴食: 携带的龙系技能获得迅捷。</t>
+    <t>暴食：携带的龙系技能获得迅捷。</t>
   </si>
   <si>
     <t>波多西</t>
@@ -537,19 +526,19 @@
     <t>机械 / 地</t>
   </si>
   <si>
-    <t>定向精炼: 己方精灵每使用1次防御技能,自己入场时机械系和地面系技能威力+10%。</t>
-  </si>
-  <si>
-    <t>里拉鲲</t>
-  </si>
-  <si>
-    <t>吟游之弦: 赋予的印记不会替换其他印记,而是同时生效。</t>
+    <t>定向精炼：己方精灵每使用1次防御技能，自己入场时机械系和地面系技能威力+10%。</t>
+  </si>
+  <si>
+    <t>里拉鳐</t>
+  </si>
+  <si>
+    <t>吟游之弦：赋予的印记不会替换其他印记，而是同时生效。</t>
   </si>
   <si>
     <t>烈火守护</t>
   </si>
   <si>
-    <t>蒸汽膨胀: 己方精灵每使用1次火系技能,自己入场时获得全技能威力+10。</t>
+    <t>蒸汽膨胀：己方精灵每使用1次火系技能，自己入场时获得全技能威力+10。</t>
   </si>
   <si>
     <t>恶魔红钻</t>
@@ -558,7 +547,7 @@
     <t>虫 / 恶</t>
   </si>
   <si>
-    <t>振奋虫心: 主动击败敌方后,己方队伍获得5次随机奉献。</t>
+    <t>振奋虫心：主动击败敌方后，己方队伍获得5次随机奉献。</t>
   </si>
   <si>
     <t>寒音蛇</t>
@@ -567,7 +556,7 @@
     <t>萌 / 毒</t>
   </si>
   <si>
-    <t>拨浪鼓: 己方精灵每使用1次状态技能,自己入场时毒系和萌系技能威力+10。</t>
+    <t>拨浪鼓：己方精灵每使用1次状态技能，自己入场时毒系和萌系技能威力+10。</t>
   </si>
   <si>
     <t>迷迷箱怪</t>
@@ -576,19 +565,19 @@
     <t>机械 / 幻</t>
   </si>
   <si>
-    <t>虚假宝箱: 自己力竭时,敌方获得攻防+20%。</t>
+    <t>虚假宝箱：自己力竭时，敌方获得攻防+20%。</t>
   </si>
   <si>
     <t>荆棘电环</t>
   </si>
   <si>
-    <t>防过载保护: 每次行动后脱离。</t>
+    <t>防过载保护：每次行动后脱离。</t>
   </si>
   <si>
     <t>酷拉</t>
   </si>
   <si>
-    <t>噼啪!: 入场后首次行动,所选技能使用次数+1。</t>
+    <t>噼啪！：入场后首次行动，所选技能使用次数+1。</t>
   </si>
   <si>
     <t>伊兰亚龙</t>
@@ -597,16 +586,16 @@
     <t>龙</t>
   </si>
   <si>
-    <t>嫉妒: 蓄力状态下,可以使用任一携带技能。</t>
-  </si>
-  <si>
-    <t>馒尾兽</t>
+    <t>嫉妒：蓄力状态下，可以使用任一携带技能。</t>
+  </si>
+  <si>
+    <t>鳗尾兽</t>
   </si>
   <si>
     <t>地 / 草</t>
   </si>
   <si>
-    <t>铃兰晚钟: 首次入场时,失去自己一半的当前生命。</t>
+    <t>铃兰晚钟：首次入场时，失去自己一半的当前生命。</t>
   </si>
   <si>
     <t>梦想三三</t>
@@ -615,7 +604,7 @@
     <t>萌</t>
   </si>
   <si>
-    <t>鼓气: 使用能耗为3的技能时,获得攻防+20%。</t>
+    <t>鼓气：使用能耗为3的技能时，获得攻防+20%。</t>
   </si>
   <si>
     <t>白发路路</t>
@@ -624,19 +613,19 @@
     <t>草 / 萌</t>
   </si>
   <si>
-    <t>营养液泡: 获得增益时,额外获得层数+2。</t>
+    <t>营养液泡：获得增益时，额外获得层数+2。</t>
   </si>
   <si>
     <t>流浪鼠</t>
   </si>
   <si>
-    <t>奔波命: 使用防御技能后,回合结束时脱离。</t>
+    <t>奔波命：使用防御技能后，回合结束时脱离。</t>
   </si>
   <si>
     <t>魔力猫</t>
   </si>
   <si>
-    <t>氧循环: 使用草系技能后,回复10%生命。</t>
+    <t>氧循环：使用草系技能后，回复10%生命。</t>
   </si>
   <si>
     <t>岚鸟</t>
@@ -645,31 +634,31 @@
     <t>翼</t>
   </si>
   <si>
-    <t>顺风: 若先于敌方攻击,本次技能威力+50%。</t>
+    <t>顺风：若先于敌方攻击，本次技能威力+50%。</t>
   </si>
   <si>
     <t>火神</t>
   </si>
   <si>
-    <t>助燃: 使用火系技能后,获得双攻+20%。</t>
+    <t>助燃：使用火系技能后，获得双攻+20%。</t>
   </si>
   <si>
     <t>水灵</t>
   </si>
   <si>
-    <t>浸润: 使用水系技能后,全技能能耗-1。</t>
+    <t>浸润：使用水系技能后，全技能能耗-1。</t>
   </si>
   <si>
     <t>水泡壳</t>
   </si>
   <si>
-    <t>缩壳: 携带的防御技能能耗-2。</t>
+    <t>缩壳：携带的防御技能能耗-2。</t>
   </si>
   <si>
     <t>花影羚羊</t>
   </si>
   <si>
-    <t>碰瓷: 自己使用恶系技能后,敌方失去2能量。</t>
+    <t>碰瓷：自己使用恶系技能后，敌方失去2能量。</t>
   </si>
   <si>
     <t>幻影灵菇</t>
@@ -678,19 +667,19 @@
     <t>幽 / 草</t>
   </si>
   <si>
-    <t>毒蘑菇: 回合结束时,偷取敌方场上所有精灵1能量。</t>
+    <t>毒蘑菇：回合结束时，偷取敌方场上所有精灵1能量。</t>
   </si>
   <si>
     <t>石冠王蜥</t>
   </si>
   <si>
-    <t>刺肤: 每受到1次攻击,对攻击自己的精灵造成50威力物理伤害。</t>
+    <t>刺肤：每受到1次攻击，对攻击自己的精灵造成50威力物理伤害。</t>
   </si>
   <si>
     <t>布克棱岩</t>
   </si>
   <si>
-    <t>地脉: 初始能量为0,入场前己方精灵每放1次地系技能,回复3能量。</t>
+    <t>地脉：初始能量为0，入场前己方精灵每放1次地系技能，回复3能量。</t>
   </si>
   <si>
     <t>叮叮恶魔</t>
@@ -699,7 +688,7 @@
     <t>恶 / 翼</t>
   </si>
   <si>
-    <t>渴求: 入场时获得50%吸血。</t>
+    <t>渴求：入场时获得50%吸血。</t>
   </si>
   <si>
     <t>化蝶</t>
@@ -708,19 +697,19 @@
     <t>虫 / 萌</t>
   </si>
   <si>
-    <t>化茧: 受到致命伤害时,获得1层硬化,并免疫此次伤害。</t>
+    <t>化茧：受到致命伤害时，获得1层硬化，并免疫此次伤害。</t>
   </si>
   <si>
     <t>卡瓦重</t>
   </si>
   <si>
-    <t>诈死: 自己力竭时,少损失1点魔力。</t>
+    <t>诈死：自己力竭时，少损失1点魔力。</t>
   </si>
   <si>
     <t>幽影树</t>
   </si>
   <si>
-    <t>小偷小摸: 入场时偷取所有敌方精灵2能量。</t>
+    <t>小偷小摸：入场时偷取所有敌方精灵2能量。</t>
   </si>
   <si>
     <t>卷胡巨獭</t>
@@ -729,7 +718,7 @@
     <t>普通 / 水</t>
   </si>
   <si>
-    <t>保守派: 总技能能耗小于4时,自己获得双防+80%。</t>
+    <t>保守派：总技能能耗小于4时，自己获得双防+80%。</t>
   </si>
   <si>
     <t>晶石蜗</t>
@@ -738,25 +727,25 @@
     <t>光 / 地</t>
   </si>
   <si>
-    <t>偏振: 受到自己携带技能系列的攻击伤害-40%。</t>
+    <t>偏振：受到自己携带技能系列的攻击伤害-40%。</t>
   </si>
   <si>
     <t>奇丽花</t>
   </si>
   <si>
-    <t>养分重吸收: 回合结束时,回复3能量。</t>
+    <t>养分重吸收：回合结束时，回复3能量。</t>
   </si>
   <si>
     <t>梦悠悠</t>
   </si>
   <si>
-    <t>做噩梦: 敌方精灵离场后,更换入场的精灵失去3能量。</t>
+    <t>做噩梦：敌方精灵离场后，更换入场的精灵失去3能量。</t>
   </si>
   <si>
     <t>音速犬</t>
   </si>
   <si>
-    <t>专注力: 入场首回合,获得物攻+100%。</t>
+    <t>专注力：入场首回合，获得物攻+100%。</t>
   </si>
   <si>
     <t>蹦床松鼠</t>
@@ -765,19 +754,19 @@
     <t>普通</t>
   </si>
   <si>
-    <t>囤积: 每有1能量,获得双防+10%。</t>
+    <t>囤积：每有1能量，获得双防+10%。</t>
   </si>
   <si>
     <t>嘟嘟锅</t>
   </si>
   <si>
-    <t>复方汤剂: 回合结束时,中毒效果触发次数+1。</t>
+    <t>复方汤剂：回合结束时，中毒效果触发次数+1。</t>
   </si>
   <si>
     <t>幽冥眼</t>
   </si>
   <si>
-    <t>惊吓: 能量等于0的精灵,无法对自己造成伤害。</t>
+    <t>惊吓：能量等于0的精灵，无法对自己造成伤害。</t>
   </si>
   <si>
     <t>兽花蕾</t>
@@ -786,13 +775,13 @@
     <t>光 / 草</t>
   </si>
   <si>
-    <t>稀兽花宝: 根据自己的血脉,入场时获得不同效果。</t>
+    <t>稀兽花宝：根据自己的血脉，入场时获得不同效果。</t>
   </si>
   <si>
     <t>巨噬针鼹</t>
   </si>
   <si>
-    <t>壮胆: 队伍存在虫系精灵,自己获得双攻+50%。</t>
+    <t>壮胆：队伍存在虫系精灵，自己获得双攻+50%。</t>
   </si>
   <si>
     <t>蹦蹦花</t>
@@ -801,43 +790,43 @@
     <t>草 / 毒</t>
   </si>
   <si>
-    <t>生物碱: 使用草系技能时,敌方获得2层中毒。</t>
+    <t>生物碱：使用草系技能时，敌方获得2层中毒。</t>
   </si>
   <si>
     <t>电球咩咩</t>
   </si>
   <si>
-    <t>快充: 离场时回复10能量。</t>
+    <t>快充：离场时回复10能量。</t>
   </si>
   <si>
     <t>蒲公英娃娃</t>
   </si>
   <si>
-    <t>勇敢: 携带的能耗大于3的技能,威力+40%。</t>
+    <t>勇敢：携带的能耗大于3的技能，威力+40%。</t>
   </si>
   <si>
     <t>菊花梨</t>
   </si>
   <si>
-    <t>无忧无虑: 可获得的弱化层数不受限制。</t>
+    <t>无忧无虑：可获得的弱化层数不受限制。</t>
   </si>
   <si>
     <t>伊贝粉粉</t>
   </si>
   <si>
-    <t>腐蚀循环: 每回复1能量,同时回复5%生命。</t>
+    <t>腐蚀循环：每回复1能量，同时回复5%生命。</t>
   </si>
   <si>
     <t>瞌睡王</t>
   </si>
   <si>
-    <t>慢热型: 初始能量为0,入场前己方精灵每成功应对1次,回复5能量。</t>
+    <t>慢热型：初始能量为0，入场前己方精灵每成功应对1次，回复5能量。</t>
   </si>
   <si>
     <t>千棘盔</t>
   </si>
   <si>
-    <t>溶解扩散: 每携带1个毒素技能进入战斗,水系技能使敌方获得1层中毒。</t>
+    <t>溶解扩散：每携带1个毒素技能进入战斗，水系技能使敌方获得1层中毒。</t>
   </si>
   <si>
     <t>翠顶夫人</t>
@@ -846,22 +835,19 @@
     <t>翼 / 水</t>
   </si>
   <si>
-    <t>洁癖: 离场后,自己的增益和减益会被更换入场的精灵继承。</t>
+    <t>洁癖：离场后，自己的增益和减益会被更换入场的精灵继承。</t>
   </si>
   <si>
     <t>星光狮</t>
   </si>
   <si>
-    <t>电流刺激: 携带的攻击技能获得迸发:威力+40。</t>
-  </si>
-  <si>
     <t>花魁蜂后</t>
   </si>
   <si>
     <t>虫 / 翼</t>
   </si>
   <si>
-    <t>虫群鼓舞: 队伍中每有1只其他的虫系精灵,自己入场时获得攻速+10%。</t>
+    <t>虫群鼓舞：队伍中每有1只其他的虫系精灵，自己入场时获得攻速+10%。</t>
   </si>
   <si>
     <t>朔夜伊芙</t>
@@ -870,7 +856,7 @@
     <t>恶</t>
   </si>
   <si>
-    <t>嫁祸: 自己每失去25%生命,连击数+2。</t>
+    <t>嫁祸：自己每失去25%生命，连击数+2。</t>
   </si>
   <si>
     <t>黑羽夫人</t>
@@ -879,13 +865,13 @@
     <t>翼 / 恶</t>
   </si>
   <si>
-    <t>贪婪: 敌方精灵离场后,其增益和减益会被更换入场的精灵继承。</t>
+    <t>贪婪：敌方精灵离场后，其增益和减益会被更换入场的精灵继承。</t>
   </si>
   <si>
     <t>锤头鹳</t>
   </si>
   <si>
-    <t>快锤: 携带的能耗小于3的技能,获得迅捷。</t>
+    <t>快锤：携带的能耗小于3的技能，获得迅捷。</t>
   </si>
   <si>
     <t>魔草巫灵</t>
@@ -894,13 +880,13 @@
     <t>草 / 幻</t>
   </si>
   <si>
-    <t>木桶戏法: 离场后,更换入场的精灵以木桶状态登场。</t>
+    <t>木桶戏法：离场后，更换入场的精灵以木桶状态登场。</t>
   </si>
   <si>
     <t>记忆石</t>
   </si>
   <si>
-    <t>不移: 携带的无额外效果的攻击技能,威力+30%。</t>
+    <t>不移：携带的无额外效果的攻击技能，威力+30%。</t>
   </si>
   <si>
     <t>罗隐</t>
@@ -909,7 +895,7 @@
     <t>地 / 恶</t>
   </si>
   <si>
-    <t>石头大餐: 能量不足时,消耗5%生命,代替1能量。</t>
+    <t>石头大餐：能量不足时，消耗5%生命，代替1能量。</t>
   </si>
   <si>
     <t>咔咔鸟</t>
@@ -918,7 +904,7 @@
     <t>翼 / 普通</t>
   </si>
   <si>
-    <t>咔咔冲刺: 若先于敌方行动,行动后获得连击数+1。</t>
+    <t>咔咔冲刺：若先于敌方行动，行动后获得连击数+1。</t>
   </si>
   <si>
     <t>花衣蝶</t>
@@ -927,7 +913,7 @@
     <t>虫 / 草</t>
   </si>
   <si>
-    <t>花精灵: 回合结束时,己方队伍获得1次随机奉献。</t>
+    <t>花精灵：回合结束时，己方队伍获得1次随机奉献。</t>
   </si>
   <si>
     <t>魔眷鸟</t>
@@ -936,7 +922,7 @@
     <t>萌 / 翼</t>
   </si>
   <si>
-    <t>自由飘: 自己每有1层萌化,获得连击数+2。</t>
+    <t>自由飘：自己每有1层萌化，获得连击数+2。</t>
   </si>
   <si>
     <t>彩蝶鲨</t>
@@ -945,7 +931,7 @@
     <t>水 / 翼</t>
   </si>
   <si>
-    <t>水翼推进: 己方精灵每使用1次水系技能,自己入场时获得全技能能耗-1。</t>
+    <t>水翼推进：己方精灵每使用1次水系技能，自己入场时获得全技能能耗-1。</t>
   </si>
   <si>
     <t>巨灵石</t>
@@ -954,7 +940,7 @@
     <t>地 / 幽</t>
   </si>
   <si>
-    <t>石天平: 若使用技能能耗高于敌方,回合结束敌方失去能耗之差的能量。</t>
+    <t>石天平：若使用技能能耗高于敌方，回合结束敌方失去能耗之差的能量。</t>
   </si>
   <si>
     <t>仪式巨像</t>
@@ -963,13 +949,13 @@
     <t>地 / 幻</t>
   </si>
   <si>
-    <t>观星: 敌方每有1层星图印记,自己的地系技能威力+15%。</t>
+    <t>观星：敌方每有1层星图印记，自己的地系技能威力+15%。</t>
   </si>
   <si>
     <t>白金独角兽</t>
   </si>
   <si>
-    <t>目空: 携带的非光系技能,威力+25%。</t>
+    <t>目空：携带的非光系技能，威力+25%。</t>
   </si>
   <si>
     <t>风滚暮虫</t>
@@ -978,13 +964,10 @@
     <t>普通 / 虫</t>
   </si>
   <si>
-    <t>共鸣: 携带的「虫鸣」技能威力+20。</t>
-  </si>
-  <si>
     <t>黑猫巫师</t>
   </si>
   <si>
-    <t>预警: 若敌方技能能够击败自己,回合开始时自己获得速度+50。</t>
+    <t>预警：若敌方技能能够击败自己，回合开始时自己获得速度+50。</t>
   </si>
   <si>
     <t>影狸</t>
@@ -993,7 +976,7 @@
     <t>幽 / 毒</t>
   </si>
   <si>
-    <t>下黑手: 敌方精灵离场后,更换入场的精灵获得5层中毒。</t>
+    <t>下黑手：敌方精灵离场后，更换入场的精灵获得5层中毒。</t>
   </si>
   <si>
     <t>古啦多</t>
@@ -1002,19 +985,19 @@
     <t>毒 / 地</t>
   </si>
   <si>
-    <t>毒牙: 使敌方获得中毒时,也会使其获得魔攻和魔防-40%。</t>
+    <t>毒牙：使敌方获得中毒时，也会使其获得魔攻和魔防-40%。</t>
   </si>
   <si>
     <t>怖哭菇</t>
   </si>
   <si>
-    <t>吸积盘: 回合结束时,敌方获得2层星痕印记。</t>
+    <t>吸积盘：回合结束时，敌方获得2层星痕印记。</t>
   </si>
   <si>
     <t>恶魔狼</t>
   </si>
   <si>
-    <t>悲悯: 己方队伍中每有1只力竭的精灵,自己获得双攻+30%。</t>
+    <t>悲悯：己方队伍中每有1只力竭的精灵，自己获得双攻+30%。</t>
   </si>
   <si>
     <t>电企鹅</t>
@@ -1023,13 +1006,10 @@
     <t>冰 / 电</t>
   </si>
   <si>
-    <t>超负荷: 攻击技能获得迸发:敌方获得全技能能耗+1。</t>
-  </si>
-  <si>
     <t>雪巨人</t>
   </si>
   <si>
-    <t>打雪仗: 初始能量为0,入场前己方精灵每放1次冰系技能,回复3能量。</t>
+    <t>打雪仗：初始能量为0，入场前己方精灵每放1次冰系技能，回复3能量。</t>
   </si>
   <si>
     <t>獠牙猪</t>
@@ -1038,13 +1018,13 @@
     <t>冰 / 地</t>
   </si>
   <si>
-    <t>冻土: 每携带1个冰系技能进入战斗,地系技能威力+10%。</t>
+    <t>冻土：每携带1个冰系技能进入战斗，地系技能威力+10%。</t>
   </si>
   <si>
     <t>雪灵</t>
   </si>
   <si>
-    <t>冰封: 在场时,敌方全技能能耗+1。</t>
+    <t>冰封：在场时，敌方全技能能耗+1。</t>
   </si>
   <si>
     <t>雪影娃娃</t>
@@ -1053,13 +1033,13 @@
     <t>冰 / 萌</t>
   </si>
   <si>
-    <t>捉迷藏: 使敌方获得冻结时,也会使其获得全技能能耗+1。</t>
+    <t>捉迷藏：使敌方获得冻结时，也会使其获得全技能能耗+1。</t>
   </si>
   <si>
     <t>权杖-V</t>
   </si>
   <si>
-    <t>机械要式: 自己携带的技能每回合位置变化时,该技能能耗-1。</t>
+    <t>机械要式：自己携带的技能每回合位置变化时，该技能能耗-1。</t>
   </si>
   <si>
     <t>尖嘴狐仙</t>
@@ -1068,13 +1048,13 @@
     <t>火 / 冰</t>
   </si>
   <si>
-    <t>灵魂灼伤: 冰系技能能使敌方获得4层灼烧,火系技能能使敌方获得2层冻结。</t>
+    <t>灵魂灼伤：冰系技能能使敌方获得4层灼烧，火系技能能使敌方获得2层冻结。</t>
   </si>
   <si>
     <t>圣羽翼王</t>
   </si>
   <si>
-    <t>飓风: 对本精灵的技能,若其他翼系精灵携带相同技能,则获得迅捷。被敌方精灵击败时,自己额外损失1点魔力。</t>
+    <t>飓风：对本精灵的技能，若其他翼系精灵携带相同技能，则获得迅捷。被敌方精灵击败时，自己额外损失1点魔力。</t>
   </si>
   <si>
     <t>针叶巡林</t>
@@ -1083,13 +1063,13 @@
     <t>草 / 武</t>
   </si>
   <si>
-    <t>野性感官: 应对成功后,下次行动先手+1。</t>
+    <t>野性感官：应对成功后，下次行动先手+1。</t>
   </si>
   <si>
     <t>炽心勇狮</t>
   </si>
   <si>
-    <t>圣火骑士: 应对成功后,下次攻击威力翻倍。</t>
+    <t>圣火骑士：应对成功后，下次攻击威力翻倍。</t>
   </si>
   <si>
     <t>游蛇魔使</t>
@@ -1098,13 +1078,13 @@
     <t>水 / 武</t>
   </si>
   <si>
-    <t>思维之盾: 应对成功后,下次行动技能能耗-5。</t>
+    <t>思维之盾：应对成功后，下次行动技能能耗-5。</t>
   </si>
   <si>
     <t>公平鸽</t>
   </si>
   <si>
-    <t>衡量: 入场时,复制敌方的增益。在场时,若敌方获得增益自己也会获得。</t>
+    <t>衡量：入场时，复制敌方的增益。在场时，若敌方获得增益自己也会获得。</t>
   </si>
   <si>
     <t>怒目怂猫</t>
@@ -1113,13 +1093,13 @@
     <t>武</t>
   </si>
   <si>
-    <t>威慑: 打断敌方时,被打断的技能进入2回合冷却。</t>
+    <t>威慑：打断敌方时，被打断的技能进入2回合冷却。</t>
   </si>
   <si>
     <t>皇家狮鹫</t>
   </si>
   <si>
-    <t>乘风连击: 使用翼系技能后,获得连击数+1。</t>
+    <t>乘风连击：使用翼系技能后，获得连击数+1。</t>
   </si>
   <si>
     <t>芋香巨角蛛</t>
@@ -1128,7 +1108,7 @@
     <t>虫 / 毒</t>
   </si>
   <si>
-    <t>毒腺: 使用能耗小于等于1的技能时,敌方获得4层中毒。</t>
+    <t>毒腺：使用能耗小于等于1的技能时，敌方获得4层中毒。</t>
   </si>
   <si>
     <t>嗜波螺</t>
@@ -1137,25 +1117,25 @@
     <t>地 / 水</t>
   </si>
   <si>
-    <t>消波块: 每携带1个水系技能进入战斗,地系技能能耗-1。</t>
+    <t>消波块：每携带1个水系技能进入战斗，地系技能能耗-1。</t>
   </si>
   <si>
     <t>九幽菇</t>
   </si>
   <si>
-    <t>多人宿舍: 自己的能量可以超过能量上限。</t>
+    <t>多人宿舍：自己的能量可以超过能量上限。</t>
   </si>
   <si>
     <t>斑枭</t>
   </si>
   <si>
-    <t>逐魂鸟: 能耗小于等于1的攻击技能,无法对自己造成伤害。</t>
+    <t>逐魂鸟：能耗小于等于1的攻击技能，无法对自己造成伤害。</t>
   </si>
   <si>
     <t>卷毛鸭</t>
   </si>
   <si>
-    <t>得寸进尺: 天气为雨天,或处于其他水系环境中时,获得双攻+100%。</t>
+    <t>得寸进尺：天气为雨天，或处于其他水系环境中时，获得双攻+100%。</t>
   </si>
   <si>
     <t>海豹船长</t>
@@ -1164,22 +1144,19 @@
     <t>武 / 水</t>
   </si>
   <si>
-    <t>身经百炼: 己方精灵每应对1次,自己入场时水系和武系技能威力+20%。</t>
+    <t>身经百炼：己方精灵每应对1次，自己入场时水系和武系技能威力+20%。</t>
   </si>
   <si>
     <t>圆号鱼</t>
   </si>
   <si>
-    <t>泛音列: 使用状态技能后,敌方获得「聒噪」技能的效果,持续3回合。</t>
-  </si>
-  <si>
     <t>卡洛儿</t>
   </si>
   <si>
     <t>水 / 萌</t>
   </si>
   <si>
-    <t>守护者: 己方其他精灵每有1层弱化,自己入场时全技能能耗-1。</t>
+    <t>守护者：己方其他精灵每有1层弱化，自己入场时全技能能耗-1。</t>
   </si>
   <si>
     <t>棋骑士</t>
@@ -1188,58 +1165,76 @@
     <t>武 / 地</t>
   </si>
   <si>
-    <t>腾挪: 攻击技能应对1次后,回满状态,变为棋骑后。</t>
+    <t>腾挪：攻击技能应对1次后，回满状态，变为棋骑后。</t>
   </si>
   <si>
     <t>棋齐垒</t>
   </si>
   <si>
-    <t>保卫: 防御技能应对2次后,回满状态,变为棋骑后。</t>
+    <t>保卫：防御技能应对2次后，回满状态，变为棋骑后。</t>
   </si>
   <si>
     <t>棋祈督</t>
   </si>
   <si>
-    <t>好象坏象: 状态技能应对1次后,回满状态,变为棋骑后。</t>
+    <t>好象坏象：状态技能应对1次后，回满状态，变为棋骑后。</t>
   </si>
   <si>
     <t>棋绮后</t>
   </si>
   <si>
-    <t>渗透: 己方精灵每使用1次武系或地系技能,自己入场时获得攻防+5%。</t>
+    <t>渗透：己方精灵每使用1次武系或地系技能，自己入场时获得攻防+5%。</t>
   </si>
   <si>
     <t>火羽</t>
   </si>
   <si>
-    <t>火/翼</t>
-  </si>
-  <si>
-    <t>急性子:每次连击赋予敌方2层灼烧。</t>
+    <t>急性子：每次连击赋予敌方2层灼烧。</t>
   </si>
   <si>
     <t>凡鹰</t>
   </si>
   <si>
-    <t>先锋:进入战斗后普通系技能变为翼系。</t>
+    <t>先锋：进入战斗后普通系技能变为翼系。</t>
   </si>
   <si>
     <t>格斗小八</t>
   </si>
   <si>
-    <t>格斗小八:入场时,若敌方本回合换宠,全属性提升100%。</t>
+    <t>格斗小八：入场时，若敌方本回合换宠，全属性提升100%。</t>
   </si>
   <si>
     <t>格斗小六</t>
   </si>
   <si>
-    <t>马步:状态技能应对成功时,获得10点能量</t>
+    <t>马步：状态技能应对成功时，获得10点能量。</t>
   </si>
   <si>
     <t>卡拉波斯</t>
   </si>
   <si>
-    <t>悬一线:首次受到致命伤害时,保留1生命值,眩晕敌方一回合。</t>
+    <t>悬一线：首次受到致命伤害时，保留1生命值，眩晕敌方一回合。</t>
+  </si>
+  <si>
+    <t>火 / 翼</t>
+  </si>
+  <si>
+    <t>生物电：携带的电系技能获得迸发：能耗-2。</t>
+  </si>
+  <si>
+    <t>电流刺激：携带的攻击技能获得迸发：威力+40。</t>
+  </si>
+  <si>
+    <t>超负荷：攻击技能获得迸发：敌方获得全技能能耗+1。</t>
+  </si>
+  <si>
+    <t>搜刮：敌方每使用1次【聚能】技能或更换精灵，自己入场时获得魔攻+20%。</t>
+  </si>
+  <si>
+    <t>共鸣：携带的【虫鸣】技能威力+20。</t>
+  </si>
+  <si>
+    <t>泛音列：使用状态技能后，敌方获得【聒噪】技能的效果，持续3回合。</t>
   </si>
 </sst>
 </file>
@@ -1589,7 +1584,7 @@
     <col min="10" max="10" width="98.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1621,7 +1616,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1653,7 +1648,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
@@ -1685,7 +1680,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
@@ -1717,7 +1712,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>19</v>
       </c>
@@ -1749,7 +1744,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>22</v>
       </c>
@@ -1781,7 +1776,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>25</v>
       </c>
@@ -1810,15 +1805,15 @@
         <v>80</v>
       </c>
       <c r="J7" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="B8" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>29</v>
       </c>
       <c r="C8" s="1">
         <v>579</v>
@@ -1842,15 +1837,15 @@
         <v>100</v>
       </c>
       <c r="J8" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="B9" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>32</v>
       </c>
       <c r="C9" s="1">
         <v>592</v>
@@ -1874,15 +1869,15 @@
         <v>115</v>
       </c>
       <c r="J9" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+      <c r="B10" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="C10" s="1">
         <v>586</v>
@@ -1906,15 +1901,15 @@
         <v>80</v>
       </c>
       <c r="J10" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+      <c r="B11" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>38</v>
       </c>
       <c r="C11" s="1">
         <v>626</v>
@@ -1938,15 +1933,15 @@
         <v>105</v>
       </c>
       <c r="J11" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+      <c r="B12" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="C12" s="1">
         <v>509</v>
@@ -1970,15 +1965,15 @@
         <v>100</v>
       </c>
       <c r="J12" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+      <c r="B13" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>44</v>
       </c>
       <c r="C13" s="1">
         <v>564</v>
@@ -2002,15 +1997,15 @@
         <v>120</v>
       </c>
       <c r="J13" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
+      <c r="B14" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="C14" s="1">
         <v>562</v>
@@ -2034,15 +2029,15 @@
         <v>120</v>
       </c>
       <c r="J14" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
+      <c r="B15" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="C15" s="1">
         <v>545</v>
@@ -2066,15 +2061,15 @@
         <v>120</v>
       </c>
       <c r="J15" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
+      <c r="B16" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>53</v>
       </c>
       <c r="C16" s="1">
         <v>612</v>
@@ -2098,15 +2093,15 @@
         <v>110</v>
       </c>
       <c r="J16" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
+      <c r="B17" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>56</v>
       </c>
       <c r="C17" s="1">
         <v>569</v>
@@ -2130,15 +2125,15 @@
         <v>115</v>
       </c>
       <c r="J17" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
+      <c r="B18" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="C18" s="1">
         <v>650</v>
@@ -2162,15 +2157,15 @@
         <v>95</v>
       </c>
       <c r="J18" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
+      <c r="B19" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>62</v>
       </c>
       <c r="C19" s="1">
         <v>658</v>
@@ -2194,15 +2189,15 @@
         <v>95</v>
       </c>
       <c r="J19" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
-        <v>64</v>
-      </c>
       <c r="B20" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C20" s="1">
         <v>608</v>
@@ -2226,15 +2221,15 @@
         <v>105</v>
       </c>
       <c r="J20" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
-        <v>66</v>
-      </c>
       <c r="B21" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C21" s="1">
         <v>619</v>
@@ -2258,15 +2253,15 @@
         <v>120</v>
       </c>
       <c r="J21" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
+      <c r="B22" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>69</v>
       </c>
       <c r="C22" s="1">
         <v>576</v>
@@ -2290,15 +2285,15 @@
         <v>115</v>
       </c>
       <c r="J22" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="B23" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C23" s="1">
         <v>565</v>
@@ -2322,15 +2317,15 @@
         <v>110</v>
       </c>
       <c r="J23" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
+      <c r="B24" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>74</v>
       </c>
       <c r="C24" s="1">
         <v>632</v>
@@ -2354,15 +2349,15 @@
         <v>100</v>
       </c>
       <c r="J24" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
+      <c r="B25" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="C25" s="1">
         <v>495</v>
@@ -2386,15 +2381,15 @@
         <v>135</v>
       </c>
       <c r="J25" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
+      <c r="B26" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="C26" s="1">
         <v>486</v>
@@ -2418,15 +2413,15 @@
         <v>85</v>
       </c>
       <c r="J26" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
+      <c r="B27" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>83</v>
       </c>
       <c r="C27" s="1">
         <v>569</v>
@@ -2450,15 +2445,15 @@
         <v>95</v>
       </c>
       <c r="J27" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
+      <c r="B28" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>86</v>
       </c>
       <c r="C28" s="1">
         <v>868</v>
@@ -2482,15 +2477,15 @@
         <v>65</v>
       </c>
       <c r="J28" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="1" t="s">
-        <v>88</v>
-      </c>
       <c r="B29" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C29" s="1">
         <v>522</v>
@@ -2514,15 +2509,15 @@
         <v>75</v>
       </c>
       <c r="J29" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="1" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
+      <c r="B30" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="C30" s="1">
         <v>576</v>
@@ -2546,15 +2541,15 @@
         <v>70</v>
       </c>
       <c r="J30" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="1" t="s">
+      <c r="B31" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>94</v>
       </c>
       <c r="C31" s="1">
         <v>604</v>
@@ -2578,15 +2573,15 @@
         <v>130</v>
       </c>
       <c r="J31" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
+      <c r="B32" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>97</v>
       </c>
       <c r="C32" s="1">
         <v>562</v>
@@ -2610,12 +2605,12 @@
         <v>110</v>
       </c>
       <c r="J32" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
         <v>98</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>11</v>
@@ -2642,15 +2637,15 @@
         <v>60</v>
       </c>
       <c r="J33" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
+      <c r="B34" s="1" t="s">
         <v>101</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>102</v>
       </c>
       <c r="C34" s="1">
         <v>588</v>
@@ -2674,15 +2669,15 @@
         <v>50</v>
       </c>
       <c r="J34" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A35" s="1" t="s">
+      <c r="B35" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="C35" s="1">
         <v>618</v>
@@ -2706,15 +2701,15 @@
         <v>145</v>
       </c>
       <c r="J35" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="1" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A36" s="1" t="s">
+      <c r="B36" s="1" t="s">
         <v>107</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>108</v>
       </c>
       <c r="C36" s="1">
         <v>605</v>
@@ -2738,15 +2733,15 @@
         <v>115</v>
       </c>
       <c r="J36" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A37" s="1" t="s">
+      <c r="B37" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="C37" s="1">
         <v>580</v>
@@ -2770,15 +2765,15 @@
         <v>95</v>
       </c>
       <c r="J37" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="1" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A38" s="1" t="s">
-        <v>113</v>
-      </c>
       <c r="B38" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C38" s="1">
         <v>661</v>
@@ -2802,15 +2797,15 @@
         <v>110</v>
       </c>
       <c r="J38" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="1" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="39" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A39" s="1" t="s">
-        <v>115</v>
-      </c>
       <c r="B39" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C39" s="1">
         <v>605</v>
@@ -2834,15 +2829,15 @@
         <v>85</v>
       </c>
       <c r="J39" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="40" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="1" t="s">
+      <c r="B40" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>118</v>
       </c>
       <c r="C40" s="1">
         <v>471</v>
@@ -2866,15 +2861,15 @@
         <v>100</v>
       </c>
       <c r="J40" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="41" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A41" s="1" t="s">
+      <c r="B41" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>121</v>
       </c>
       <c r="C41" s="1">
         <v>615</v>
@@ -2898,15 +2893,15 @@
         <v>55</v>
       </c>
       <c r="J41" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="42" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A42" s="1" t="s">
+      <c r="B42" s="1" t="s">
         <v>123</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>124</v>
       </c>
       <c r="C42" s="1">
         <v>598</v>
@@ -2930,15 +2925,15 @@
         <v>90</v>
       </c>
       <c r="J42" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="1" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="43" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A43" s="1" t="s">
+      <c r="B43" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>127</v>
       </c>
       <c r="C43" s="1">
         <v>493</v>
@@ -2962,15 +2957,15 @@
         <v>90</v>
       </c>
       <c r="J43" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="1" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="44" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A44" s="1" t="s">
+      <c r="B44" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>130</v>
       </c>
       <c r="C44" s="1">
         <v>715</v>
@@ -2994,15 +2989,15 @@
         <v>60</v>
       </c>
       <c r="J44" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="1" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="45" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A45" s="1" t="s">
+      <c r="B45" s="1" t="s">
         <v>132</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>133</v>
       </c>
       <c r="C45" s="1">
         <v>520</v>
@@ -3026,15 +3021,15 @@
         <v>125</v>
       </c>
       <c r="J45" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="46" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="1" t="s">
+      <c r="B46" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>136</v>
       </c>
       <c r="C46" s="1">
         <v>580</v>
@@ -3058,15 +3053,15 @@
         <v>95</v>
       </c>
       <c r="J46" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="47" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A47" s="1" t="s">
+      <c r="B47" s="1" t="s">
         <v>138</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>139</v>
       </c>
       <c r="C47" s="1">
         <v>646</v>
@@ -3090,15 +3085,15 @@
         <v>115</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C48" s="1">
         <v>612</v>
@@ -3122,15 +3117,15 @@
         <v>100</v>
       </c>
       <c r="J48" s="1" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C49" s="1">
         <v>611</v>
@@ -3154,15 +3149,15 @@
         <v>105</v>
       </c>
       <c r="J49" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="1" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A50" s="1" t="s">
-        <v>144</v>
-      </c>
       <c r="B50" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C50" s="1">
         <v>614</v>
@@ -3186,15 +3181,15 @@
         <v>100</v>
       </c>
       <c r="J50" s="1" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C51" s="1">
         <v>667</v>
@@ -3218,15 +3213,15 @@
         <v>125</v>
       </c>
       <c r="J51" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B52" s="1" t="s">
         <v>147</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A52" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>149</v>
       </c>
       <c r="C52" s="1">
         <v>609</v>
@@ -3250,15 +3245,15 @@
         <v>105</v>
       </c>
       <c r="J52" s="1" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B53" s="1" t="s">
         <v>150</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A53" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>152</v>
       </c>
       <c r="C53" s="1">
         <v>534</v>
@@ -3282,15 +3277,15 @@
         <v>115</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C54" s="1">
         <v>568</v>
@@ -3314,15 +3309,15 @@
         <v>90</v>
       </c>
       <c r="J54" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B55" s="1" t="s">
         <v>155</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A55" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>157</v>
       </c>
       <c r="C55" s="1">
         <v>532</v>
@@ -3346,15 +3341,15 @@
         <v>120</v>
       </c>
       <c r="J55" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B56" s="1" t="s">
         <v>158</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A56" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>160</v>
       </c>
       <c r="C56" s="1">
         <v>603</v>
@@ -3378,15 +3373,15 @@
         <v>120</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C57" s="1">
         <v>610</v>
@@ -3410,15 +3405,15 @@
         <v>110</v>
       </c>
       <c r="J57" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="1" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="58" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A58" s="1" t="s">
-        <v>163</v>
-      </c>
       <c r="B58" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C58" s="1">
         <v>607</v>
@@ -3442,15 +3437,15 @@
         <v>110</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C59" s="1">
         <v>610</v>
@@ -3474,15 +3469,15 @@
         <v>110</v>
       </c>
       <c r="J59" s="1" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C60" s="1">
         <v>513</v>
@@ -3506,15 +3501,15 @@
         <v>115</v>
       </c>
       <c r="J60" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B61" s="1" t="s">
         <v>167</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A61" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>169</v>
       </c>
       <c r="C61" s="1">
         <v>573</v>
@@ -3538,15 +3533,15 @@
         <v>50</v>
       </c>
       <c r="J61" s="1" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C62" s="1">
         <v>644</v>
@@ -3570,15 +3565,15 @@
         <v>105</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C63" s="1">
         <v>504</v>
@@ -3602,15 +3597,15 @@
         <v>65</v>
       </c>
       <c r="J63" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B64" s="1" t="s">
         <v>174</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A64" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="B64" s="1" t="s">
-        <v>176</v>
       </c>
       <c r="C64" s="1">
         <v>666</v>
@@ -3634,15 +3629,15 @@
         <v>115</v>
       </c>
       <c r="J64" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="B65" s="1" t="s">
         <v>177</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A65" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B65" s="1" t="s">
-        <v>179</v>
       </c>
       <c r="C65" s="1">
         <v>558</v>
@@ -3666,15 +3661,15 @@
         <v>100</v>
       </c>
       <c r="J65" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B66" s="1" t="s">
         <v>180</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A66" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>182</v>
       </c>
       <c r="C66" s="1">
         <v>782</v>
@@ -3698,15 +3693,15 @@
         <v>80</v>
       </c>
       <c r="J66" s="1" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C67" s="1">
         <v>557</v>
@@ -3730,15 +3725,15 @@
         <v>120</v>
       </c>
       <c r="J67" s="1" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C68" s="1">
         <v>583</v>
@@ -3762,15 +3757,15 @@
         <v>125</v>
       </c>
       <c r="J68" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B69" s="1" t="s">
         <v>187</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A69" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>189</v>
       </c>
       <c r="C69" s="1">
         <v>651</v>
@@ -3794,15 +3789,15 @@
         <v>90</v>
       </c>
       <c r="J69" s="1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B70" s="1" t="s">
         <v>190</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A70" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>192</v>
       </c>
       <c r="C70" s="1">
         <v>788</v>
@@ -3826,15 +3821,15 @@
         <v>65</v>
       </c>
       <c r="J70" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B71" s="1" t="s">
         <v>193</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A71" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="B71" s="1" t="s">
-        <v>195</v>
       </c>
       <c r="C71" s="1">
         <v>641</v>
@@ -3858,15 +3853,15 @@
         <v>110</v>
       </c>
       <c r="J71" s="1" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B72" s="1" t="s">
         <v>196</v>
-      </c>
-    </row>
-    <row r="72" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A72" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>198</v>
       </c>
       <c r="C72" s="1">
         <v>633</v>
@@ -3890,15 +3885,15 @@
         <v>95</v>
       </c>
       <c r="J72" s="1" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="73" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C73" s="1">
         <v>563</v>
@@ -3922,12 +3917,12 @@
         <v>115</v>
       </c>
       <c r="J73" s="1" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B74" s="1" t="s">
         <v>11</v>
@@ -3954,15 +3949,15 @@
         <v>55</v>
       </c>
       <c r="J74" s="1" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B75" s="1" t="s">
         <v>203</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A75" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="B75" s="1" t="s">
-        <v>205</v>
       </c>
       <c r="C75" s="1">
         <v>570</v>
@@ -3986,15 +3981,15 @@
         <v>115</v>
       </c>
       <c r="J75" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="76" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C76" s="1">
         <v>613</v>
@@ -4018,15 +4013,15 @@
         <v>130</v>
       </c>
       <c r="J76" s="1" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C77" s="1">
         <v>621</v>
@@ -4050,15 +4045,15 @@
         <v>85</v>
       </c>
       <c r="J77" s="1" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C78" s="1">
         <v>594</v>
@@ -4082,15 +4077,15 @@
         <v>75</v>
       </c>
       <c r="J78" s="1" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C79" s="1">
         <v>582</v>
@@ -4114,15 +4109,15 @@
         <v>110</v>
       </c>
       <c r="J79" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="B80" s="1" t="s">
         <v>214</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A80" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="B80" s="1" t="s">
-        <v>216</v>
       </c>
       <c r="C80" s="1">
         <v>621</v>
@@ -4146,15 +4141,15 @@
         <v>75</v>
       </c>
       <c r="J80" s="1" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="81" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C81" s="1">
         <v>572</v>
@@ -4178,15 +4173,15 @@
         <v>95</v>
       </c>
       <c r="J81" s="1" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="82" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C82" s="1">
         <v>683</v>
@@ -4210,15 +4205,15 @@
         <v>70</v>
       </c>
       <c r="J82" s="1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="B83" s="1" t="s">
         <v>221</v>
-      </c>
-    </row>
-    <row r="83" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A83" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="B83" s="1" t="s">
-        <v>223</v>
       </c>
       <c r="C83" s="1">
         <v>535</v>
@@ -4242,15 +4237,15 @@
         <v>105</v>
       </c>
       <c r="J83" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="B84" s="1" t="s">
         <v>224</v>
-      </c>
-    </row>
-    <row r="84" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A84" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="B84" s="1" t="s">
-        <v>226</v>
       </c>
       <c r="C84" s="1">
         <v>377</v>
@@ -4274,12 +4269,12 @@
         <v>100</v>
       </c>
       <c r="J84" s="1" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="85" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B85" s="1" t="s">
         <v>11</v>
@@ -4306,15 +4301,15 @@
         <v>130</v>
       </c>
       <c r="J85" s="1" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C86" s="1">
         <v>571</v>
@@ -4338,15 +4333,15 @@
         <v>80</v>
       </c>
       <c r="J86" s="1" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="B87" s="1" t="s">
         <v>231</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A87" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="B87" s="1" t="s">
-        <v>233</v>
       </c>
       <c r="C87" s="1">
         <v>595</v>
@@ -4370,15 +4365,15 @@
         <v>80</v>
       </c>
       <c r="J87" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="B88" s="1" t="s">
         <v>234</v>
-      </c>
-    </row>
-    <row r="88" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A88" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="B88" s="1" t="s">
-        <v>236</v>
       </c>
       <c r="C88" s="1">
         <v>583</v>
@@ -4402,12 +4397,12 @@
         <v>65</v>
       </c>
       <c r="J88" s="1" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="89" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B89" s="1" t="s">
         <v>11</v>
@@ -4434,12 +4429,12 @@
         <v>80</v>
       </c>
       <c r="J89" s="1" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="90" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B90" s="1" t="s">
         <v>26</v>
@@ -4466,15 +4461,15 @@
         <v>115</v>
       </c>
       <c r="J90" s="1" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="91" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C91" s="1">
         <v>562</v>
@@ -4498,15 +4493,15 @@
         <v>120</v>
       </c>
       <c r="J91" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B92" s="1" t="s">
         <v>243</v>
-      </c>
-    </row>
-    <row r="92" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A92" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="B92" s="1" t="s">
-        <v>245</v>
       </c>
       <c r="C92" s="1">
         <v>555</v>
@@ -4530,15 +4525,15 @@
         <v>80</v>
       </c>
       <c r="J92" s="1" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="93" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C93" s="1">
         <v>573</v>
@@ -4562,12 +4557,12 @@
         <v>105</v>
       </c>
       <c r="J93" s="1" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="94" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B94" s="1" t="s">
         <v>26</v>
@@ -4594,15 +4589,15 @@
         <v>115</v>
       </c>
       <c r="J94" s="1" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="B95" s="1" t="s">
         <v>250</v>
-      </c>
-    </row>
-    <row r="95" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A95" s="1" t="s">
-        <v>251</v>
-      </c>
-      <c r="B95" s="1" t="s">
-        <v>252</v>
       </c>
       <c r="C95" s="1">
         <v>513</v>
@@ -4626,15 +4621,15 @@
         <v>115</v>
       </c>
       <c r="J95" s="1" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="96" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C96" s="1">
         <v>562</v>
@@ -4658,15 +4653,15 @@
         <v>85</v>
       </c>
       <c r="J96" s="1" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="B97" s="1" t="s">
         <v>255</v>
-      </c>
-    </row>
-    <row r="97" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A97" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="B97" s="1" t="s">
-        <v>257</v>
       </c>
       <c r="C97" s="1">
         <v>580</v>
@@ -4690,15 +4685,15 @@
         <v>85</v>
       </c>
       <c r="J97" s="1" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="98" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C98" s="1">
         <v>553</v>
@@ -4722,15 +4717,15 @@
         <v>125</v>
       </c>
       <c r="J98" s="1" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="99" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C99" s="1">
         <v>642</v>
@@ -4754,15 +4749,15 @@
         <v>65</v>
       </c>
       <c r="J99" s="1" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="100" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C100" s="1">
         <v>523</v>
@@ -4786,12 +4781,12 @@
         <v>60</v>
       </c>
       <c r="J100" s="1" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="101" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B101" s="1" t="s">
         <v>11</v>
@@ -4818,15 +4813,15 @@
         <v>90</v>
       </c>
       <c r="J101" s="1" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="102" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C102" s="1">
         <v>685</v>
@@ -4850,15 +4845,15 @@
         <v>75</v>
       </c>
       <c r="J102" s="1" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="103" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C103" s="1">
         <v>545</v>
@@ -4882,15 +4877,15 @@
         <v>100</v>
       </c>
       <c r="J103" s="1" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="B104" s="1" t="s">
         <v>270</v>
-      </c>
-    </row>
-    <row r="104" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A104" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="B104" s="1" t="s">
-        <v>272</v>
       </c>
       <c r="C104" s="1">
         <v>656</v>
@@ -4914,15 +4909,15 @@
         <v>115</v>
       </c>
       <c r="J104" s="1" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="105" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C105" s="1">
         <v>617</v>
@@ -4946,15 +4941,15 @@
         <v>135</v>
       </c>
       <c r="J105" s="1" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="106" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="C106" s="1">
         <v>382</v>
@@ -4978,15 +4973,15 @@
         <v>44</v>
       </c>
       <c r="J106" s="1" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="107" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="C107" s="1">
         <v>624</v>
@@ -5010,15 +5005,15 @@
         <v>115</v>
       </c>
       <c r="J107" s="1" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="108" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="C108" s="1">
         <v>652</v>
@@ -5042,15 +5037,15 @@
         <v>120</v>
       </c>
       <c r="J108" s="1" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="109" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C109" s="1">
         <v>511</v>
@@ -5074,15 +5069,15 @@
         <v>105</v>
       </c>
       <c r="J109" s="1" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="110" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="C110" s="1">
         <v>592</v>
@@ -5106,15 +5101,15 @@
         <v>90</v>
       </c>
       <c r="J110" s="1" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="111" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C111" s="1">
         <v>607</v>
@@ -5138,15 +5133,15 @@
         <v>70</v>
       </c>
       <c r="J111" s="1" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="112" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="C112" s="1">
         <v>601</v>
@@ -5170,15 +5165,15 @@
         <v>75</v>
       </c>
       <c r="J112" s="1" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="113" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C113" s="1">
         <v>631</v>
@@ -5202,15 +5197,15 @@
         <v>120</v>
       </c>
       <c r="J113" s="1" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="114" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="C114" s="1">
         <v>539</v>
@@ -5234,15 +5229,15 @@
         <v>100</v>
       </c>
       <c r="J114" s="1" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="115" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="C115" s="1">
         <v>551</v>
@@ -5266,15 +5261,15 @@
         <v>135</v>
       </c>
       <c r="J115" s="1" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="116" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="C116" s="1">
         <v>579</v>
@@ -5298,15 +5293,15 @@
         <v>125</v>
       </c>
       <c r="J116" s="1" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="117" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="117" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="C117" s="1">
         <v>584</v>
@@ -5330,15 +5325,15 @@
         <v>95</v>
       </c>
       <c r="J117" s="1" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="118" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C118" s="1">
         <v>610</v>
@@ -5362,15 +5357,15 @@
         <v>85</v>
       </c>
       <c r="J118" s="1" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="119" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C119" s="1">
         <v>595</v>
@@ -5394,15 +5389,15 @@
         <v>105</v>
       </c>
       <c r="J119" s="1" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="120" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="C120" s="1">
         <v>542</v>
@@ -5426,15 +5421,15 @@
         <v>120</v>
       </c>
       <c r="J120" s="1" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="121" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="1" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C121" s="1">
         <v>662</v>
@@ -5458,15 +5453,15 @@
         <v>70</v>
       </c>
       <c r="J121" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="122" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="1" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="C122" s="1">
         <v>616</v>
@@ -5490,15 +5485,15 @@
         <v>130</v>
       </c>
       <c r="J122" s="1" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="123" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="C123" s="1">
         <v>591</v>
@@ -5522,12 +5517,12 @@
         <v>90</v>
       </c>
       <c r="J123" s="1" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="124" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A124" s="1" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="B124" s="1" t="s">
         <v>14</v>
@@ -5554,15 +5549,15 @@
         <v>60</v>
       </c>
       <c r="J124" s="1" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="125" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="C125" s="1">
         <v>548</v>
@@ -5586,15 +5581,15 @@
         <v>120</v>
       </c>
       <c r="J125" s="1" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="126" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="C126" s="1">
         <v>583</v>
@@ -5618,15 +5613,15 @@
         <v>125</v>
       </c>
       <c r="J126" s="1" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="127" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C127" s="1">
         <v>718</v>
@@ -5650,15 +5645,15 @@
         <v>60</v>
       </c>
       <c r="J127" s="1" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="128" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="C128" s="1">
         <v>579</v>
@@ -5682,15 +5677,15 @@
         <v>85</v>
       </c>
       <c r="J128" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="129" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C129" s="1">
         <v>643</v>
@@ -5714,15 +5709,15 @@
         <v>115</v>
       </c>
       <c r="J129" s="1" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="130" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="C130" s="1">
         <v>617</v>
@@ -5746,15 +5741,15 @@
         <v>90</v>
       </c>
       <c r="J130" s="1" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="131" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C131" s="1">
         <v>652</v>
@@ -5778,15 +5773,15 @@
         <v>75</v>
       </c>
       <c r="J131" s="1" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="132" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="132" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="C132" s="1">
         <v>580</v>
@@ -5810,15 +5805,15 @@
         <v>100</v>
       </c>
       <c r="J132" s="1" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="133" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="133" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C133" s="1">
         <v>685</v>
@@ -5842,15 +5837,15 @@
         <v>125</v>
       </c>
       <c r="J133" s="1" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="134" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="134" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="C134" s="1">
         <v>634</v>
@@ -5874,15 +5869,15 @@
         <v>105</v>
       </c>
       <c r="J134" s="1" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="135" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="135" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C135" s="1">
         <v>597</v>
@@ -5906,15 +5901,15 @@
         <v>80</v>
       </c>
       <c r="J135" s="1" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="136" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="136" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A136" s="1" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="C136" s="1">
         <v>630</v>
@@ -5938,15 +5933,15 @@
         <v>105</v>
       </c>
       <c r="J136" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="137" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="137" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C137" s="1">
         <v>649</v>
@@ -5970,15 +5965,15 @@
         <v>100</v>
       </c>
       <c r="J137" s="1" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="138" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="138" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="C138" s="1">
         <v>651</v>
@@ -6002,15 +5997,15 @@
         <v>95</v>
       </c>
       <c r="J138" s="1" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="139" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="139" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A139" s="1" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C139" s="1">
         <v>564</v>
@@ -6034,15 +6029,15 @@
         <v>120</v>
       </c>
       <c r="J139" s="1" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="140" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="140" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A140" s="1" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="C140" s="1">
         <v>506</v>
@@ -6066,15 +6061,15 @@
         <v>110</v>
       </c>
       <c r="J140" s="1" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="141" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="141" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A141" s="1" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="C141" s="1">
         <v>634</v>
@@ -6098,15 +6093,15 @@
         <v>70</v>
       </c>
       <c r="J141" s="1" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="142" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="142" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="1" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C142" s="1">
         <v>627</v>
@@ -6130,15 +6125,15 @@
         <v>70</v>
       </c>
       <c r="J142" s="1" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="143" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="143" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A143" s="1" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C143" s="1">
         <v>617</v>
@@ -6162,15 +6157,15 @@
         <v>115</v>
       </c>
       <c r="J143" s="1" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="144" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="144" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="C144" s="1">
         <v>504</v>
@@ -6194,15 +6189,15 @@
         <v>115</v>
       </c>
       <c r="J144" s="1" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="145" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="145" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A145" s="1" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="C145" s="1">
         <v>600</v>
@@ -6226,15 +6221,15 @@
         <v>100</v>
       </c>
       <c r="J145" s="1" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="146" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="146" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" s="1" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C146" s="1">
         <v>575</v>
@@ -6258,15 +6253,15 @@
         <v>105</v>
       </c>
       <c r="J146" s="1" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="147" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="147" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="1" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="C147" s="1">
         <v>619</v>
@@ -6290,15 +6285,15 @@
         <v>90</v>
       </c>
       <c r="J147" s="1" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="148" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="148" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A148" s="1" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="C148" s="1">
         <v>543</v>
@@ -6322,15 +6317,15 @@
         <v>125</v>
       </c>
       <c r="J148" s="1" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="149" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="149" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A149" s="1" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="C149" s="1">
         <v>489</v>
@@ -6354,15 +6349,15 @@
         <v>75</v>
       </c>
       <c r="J149" s="1" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="150" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="150" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="1" t="s">
-        <v>390</v>
+        <v>384</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="C150" s="1">
         <v>547</v>
@@ -6386,15 +6381,15 @@
         <v>85</v>
       </c>
       <c r="J150" s="1" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="151" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="151" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A151" s="1" t="s">
-        <v>392</v>
+        <v>386</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="C151" s="1">
         <v>508</v>
@@ -6418,15 +6413,15 @@
         <v>90</v>
       </c>
       <c r="J151" s="1" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="152" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="152" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A152" s="1" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="C152" s="1">
         <v>619</v>
@@ -6450,15 +6445,15 @@
         <v>120</v>
       </c>
       <c r="J152" s="1" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="153" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="153" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A153" s="1" t="s">
-        <v>397</v>
+        <v>390</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C153" s="1">
         <v>627</v>
@@ -6482,15 +6477,15 @@
         <v>125</v>
       </c>
       <c r="J153" s="1" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="154" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="154" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A154" s="1" t="s">
-        <v>399</v>
+        <v>392</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="C154" s="1">
         <v>565</v>
@@ -6514,15 +6509,15 @@
         <v>56</v>
       </c>
       <c r="J154" s="1" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="155" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="155" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A155" s="1" t="s">
-        <v>401</v>
+        <v>394</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="C155" s="1">
         <v>639</v>
@@ -6546,15 +6541,15 @@
         <v>150</v>
       </c>
       <c r="J155" s="1" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="156" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="156" spans="1:10" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A156" s="1" t="s">
-        <v>403</v>
+        <v>396</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="C156" s="1">
         <v>542</v>
@@ -6578,7 +6573,7 @@
         <v>100</v>
       </c>
       <c r="J156" s="1" t="s">
-        <v>404</v>
+        <v>397</v>
       </c>
     </row>
   </sheetData>

</xml_diff>